<commit_message>
Zone table list add on
</commit_message>
<xml_diff>
--- a/public/file/Retail International Economy Rates Upload Template.xlsx
+++ b/public/file/Retail International Economy Rates Upload Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\sonic_3\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0E1E9F5-D872-4747-85A7-9E32FEC49472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FC65A5-94D1-451C-A5E2-ED22CD57855B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Range Down</t>
   </si>
@@ -60,10 +60,19 @@
     <t>Range Up</t>
   </si>
   <si>
-    <t>Zone 8</t>
+    <t>Zone 1a</t>
   </si>
   <si>
-    <t>Zone 1</t>
+    <t>Zone 1b</t>
+  </si>
+  <si>
+    <t>Zone 8c</t>
+  </si>
+  <si>
+    <t>Zone 8b</t>
+  </si>
+  <si>
+    <t>Zone 8a</t>
   </si>
 </sst>
 </file>
@@ -488,14 +497,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M601"/>
+  <dimension ref="A1:P601"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" customWidth="1"/>
     <col min="2" max="2" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -503,40 +512,49 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>0.01</v>
       </c>
@@ -544,7 +562,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>0.51</v>
       </c>
@@ -552,7 +570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>1.01</v>
       </c>
@@ -560,7 +578,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>1.51</v>
       </c>
@@ -568,7 +586,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>2.0099999999999998</v>
       </c>
@@ -576,7 +594,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>2.5099999999999998</v>
       </c>
@@ -584,7 +602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>3.01</v>
       </c>
@@ -592,7 +610,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>3.51</v>
       </c>
@@ -600,7 +618,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>4.01</v>
       </c>
@@ -608,7 +626,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>4.51</v>
       </c>
@@ -616,7 +634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>5.01</v>
       </c>
@@ -624,7 +642,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>5.51</v>
       </c>
@@ -632,7 +650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>6.01</v>
       </c>
@@ -640,7 +658,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>6.51</v>
       </c>
@@ -648,7 +666,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>7.01</v>
       </c>

</xml_diff>